<commit_message>
Release prompt-only storyboard workflow
</commit_message>
<xml_diff>
--- a/skills/make-ai-comic-drama/assets/AI漫剧生产信息表模板.xlsx
+++ b/skills/make-ai-comic-drama/assets/AI漫剧生产信息表模板.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="项目总览" sheetId="1" r:id="R7f279d8c731441b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="母资产总表" sheetId="2" r:id="R1bc69f3dd08c48a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="场景机位矩阵" sheetId="3" r:id="R0c841f51790844ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分镜组资产矩阵" sheetId="4" r:id="Rbf72ca30280347b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="子资产生产清单" sheetId="5" r:id="R8adeaa5cf1c4400c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="视频输入包" sheetId="6" r:id="Rfe12cf3945dc4045"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分集声音执行表" sheetId="7" r:id="R025df66a61964812"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="项目总览" sheetId="1" r:id="Rc29743e46cd54f88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="母资产总表" sheetId="2" r:id="R0c4aa6aacac4444d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="场景机位矩阵" sheetId="3" r:id="Ra1e064abff8c49aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分镜组资产矩阵" sheetId="4" r:id="R6ea3050fbebe43f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="子资产生产清单" sheetId="5" r:id="R386502bd73fa4891"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="视频输入包" sheetId="6" r:id="R9632ec59372c482b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分集声音执行表" sheetId="7" r:id="R5db84bb0c4764186"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1074,10 +1074,10 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="48" t="str">
-        <x:v>CHAR-LZ</x:v>
+        <x:v>CHAR-LM</x:v>
       </x:c>
       <x:c r="B3" s="48" t="str">
-        <x:v>林舟</x:v>
+        <x:v>李明</x:v>
       </x:c>
       <x:c r="C3" s="48" t="str">
         <x:v>CHARACTER</x:v>
@@ -1767,7 +1767,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re883f0771cc54935"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra1cba458f59f4245"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1836,7 +1836,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="48" t="str">
-        <x:v>综合训练教室</x:v>
+        <x:v>金融一班教室</x:v>
       </x:c>
       <x:c r="B3" s="48" t="str">
         <x:v>讲台向后排</x:v>
@@ -2477,7 +2477,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9848253367734237"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ae676add37a4be6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2573,19 +2573,19 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="E3" s="48" t="str">
-        <x:v>林舟、苏澄</x:v>
+        <x:v>李明、张三</x:v>
       </x:c>
       <x:c r="F3" s="48" t="str">
         <x:v>日常服/正常</x:v>
       </x:c>
       <x:c r="G3" s="48" t="str">
-        <x:v>综合训练教室</x:v>
+        <x:v>金融一班教室</x:v>
       </x:c>
       <x:c r="H3" s="48" t="str">
         <x:v>讲台向后排</x:v>
       </x:c>
       <x:c r="I3" s="48" t="str">
-        <x:v>练习长剑</x:v>
+        <x:v>黄金剑</x:v>
       </x:c>
       <x:c r="J3" s="48" t="str">
         <x:v>无</x:v>
@@ -3357,7 +3357,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a818ee4c1154775"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62fdbd0e08664302"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3438,7 +3438,7 @@
         <x:v>BLOCKING</x:v>
       </x:c>
       <x:c r="E3" s="48" t="str">
-        <x:v>林舟与苏澄双人站位</x:v>
+        <x:v>李明与张三双人站位</x:v>
       </x:c>
       <x:c r="F3" s="48" t="str">
         <x:v>锁定两人距离与朝向</x:v>
@@ -3447,7 +3447,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="H3" s="48" t="str">
-        <x:v>林舟、苏澄、综合训练教室</x:v>
+        <x:v>李明、张三、金融一班教室</x:v>
       </x:c>
       <x:c r="I3" s="48" t="str">
         <x:v>PENDING</x:v>
@@ -4070,7 +4070,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9512b59d5ea0423f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb9a955527134fa8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5089,7 +5089,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f034a4ac0c649f0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red51d8320ebc4e1a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6189,7 +6189,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd1de83d9e19844cc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R334612ed05094d19"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>